<commit_message>
Add the Order Desk: front-store orders that reduce stock
A front store sends a PC spec; the Order Desk agent (Groq with Gemini
fallback, chat memory, calculator) matches parts, checks stock and
compatibility, suggests in-stock alternatives, shows the total, and
asks for the store location after confirmation. Check Order validates
the order against the live sheet before Update Stock lowers stock_qty
and Log Order appends to the new Orders tab. The Router gets its own
memory for follow-ups, and body.mode "order" routes straight to the
Order Desk.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xa8wM77djPGNZJH4YD6QdD
</commit_message>
<xml_diff>
--- a/inventory/pc_parts_inventory.xlsx
+++ b/inventory/pc_parts_inventory.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Inventory" sheetId="1" r:id="rId1"/>
+    <sheet name="Orders" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -77494,4 +77495,35 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H2965"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>order_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>date</v>
+      </c>
+      <c r="C1" t="str">
+        <v>store_location</v>
+      </c>
+      <c r="D1" t="str">
+        <v>items</v>
+      </c>
+      <c r="E1" t="str">
+        <v>total_incl_vat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>session_id</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Order Desk keeps quoted parts on confirm; fix garbled product names
- Prepare Request: the product list header now says products talked
  about earlier may be missing from the list for the latest message
- Order Desk: on "confirm", keep the SKUs from the last summary instead
  of calling them missing (live test: it said the 5600X and RTX 4070
  were not in stock after "confirm, Bang Na branch")
- Check Order: accept SKUs written with special dashes or spaces, and
  ORDER_JSON inside code blocks or after a bold label
- build_pc_parts_sheet.js: read the CSV files as UTF-8; 59 names had
  garbled symbols. Regenerated pc_parts_inventory.xlsx (same SKUs,
  prices and stock)
- HANDOFF_PROMPT.md: live order test results

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xa8wM77djPGNZJH4YD6QdD
</commit_message>
<xml_diff>
--- a/inventory/pc_parts_inventory.xlsx
+++ b/inventory/pc_parts_inventory.xlsx
@@ -6697,7 +6697,7 @@
         <v>ZT-D40610H-10SMP</v>
       </c>
       <c r="B243" t="str">
-        <v>ZOTAC Gaming GeForce RTX 4060 Ti Twin Edge OC SPIDER-MANâ¢ Across the Spider-Verse</v>
+        <v>ZOTAC Gaming GeForce RTX 4060 Ti Twin Edge OC SPIDER-MAN™ Across the Spider-Verse</v>
       </c>
       <c r="C243" t="str">
         <v>gpu</v>
@@ -21569,7 +21569,7 @@
         <v>CMD16GX3M2A2400C11</v>
       </c>
       <c r="B815" t="str">
-        <v>Corsair Dominator Platinum Series â 16GB</v>
+        <v>Corsair Dominator Platinum Series — 16GB</v>
       </c>
       <c r="C815" t="str">
         <v>ram</v>
@@ -21647,7 +21647,7 @@
         <v>CML32GX3M4A1600C10</v>
       </c>
       <c r="B818" t="str">
-        <v>Corsair Low Profile â 32GB Dual/Quad Channel DDR3 Memory Kit</v>
+        <v>Corsair Low Profile — 32GB Dual/Quad Channel DDR3 Memory Kit</v>
       </c>
       <c r="C818" t="str">
         <v>ram</v>
@@ -21673,7 +21673,7 @@
         <v>CML4GX3M2A1600C9</v>
       </c>
       <c r="B819" t="str">
-        <v>Corsair Low Profile â 4GB Dual Channel DDR3 Memory Kit</v>
+        <v>Corsair Low Profile — 4GB Dual Channel DDR3 Memory Kit</v>
       </c>
       <c r="C819" t="str">
         <v>ram</v>
@@ -21699,7 +21699,7 @@
         <v>CML8GX3M2A1600C9R</v>
       </c>
       <c r="B820" t="str">
-        <v>Corsair Low Profile â 8GB Dual Channel DDR3 Memory Kit</v>
+        <v>Corsair Low Profile — 8GB Dual Channel DDR3 Memory Kit</v>
       </c>
       <c r="C820" t="str">
         <v>ram</v>
@@ -22141,7 +22141,7 @@
         <v>CMY16GX3M2A1600C9A</v>
       </c>
       <c r="B837" t="str">
-        <v>Corsair Pro Series â 16GB</v>
+        <v>Corsair Pro Series — 16GB</v>
       </c>
       <c r="C837" t="str">
         <v>ram</v>
@@ -22167,7 +22167,7 @@
         <v>CMY16GX3M2B2133C11</v>
       </c>
       <c r="B838" t="str">
-        <v>Corsair Pro Series â 16GB</v>
+        <v>Corsair Pro Series — 16GB</v>
       </c>
       <c r="C838" t="str">
         <v>ram</v>
@@ -22193,7 +22193,7 @@
         <v>CMY16GX3M2A2400C11R</v>
       </c>
       <c r="B839" t="str">
-        <v>Corsair Pro Series â 16GB</v>
+        <v>Corsair Pro Series — 16GB</v>
       </c>
       <c r="C839" t="str">
         <v>ram</v>
@@ -22219,7 +22219,7 @@
         <v>CMY32GX3M4A1600C9</v>
       </c>
       <c r="B840" t="str">
-        <v>Corsair Pro Series â 32GB</v>
+        <v>Corsair Pro Series — 32GB</v>
       </c>
       <c r="C840" t="str">
         <v>ram</v>
@@ -22245,7 +22245,7 @@
         <v>CMY32GX3M4A1600C9R</v>
       </c>
       <c r="B841" t="str">
-        <v>Corsair Pro Series â 32GB</v>
+        <v>Corsair Pro Series — 32GB</v>
       </c>
       <c r="C841" t="str">
         <v>ram</v>
@@ -22271,7 +22271,7 @@
         <v>CMY32GX3M4A1600C9B</v>
       </c>
       <c r="B842" t="str">
-        <v>Corsair Pro Series â 32GB</v>
+        <v>Corsair Pro Series — 32GB</v>
       </c>
       <c r="C842" t="str">
         <v>ram</v>
@@ -22297,7 +22297,7 @@
         <v>CMY8GX3M2A1600C9</v>
       </c>
       <c r="B843" t="str">
-        <v>Corsair Pro Series â 8GB</v>
+        <v>Corsair Pro Series — 8GB</v>
       </c>
       <c r="C843" t="str">
         <v>ram</v>
@@ -22323,7 +22323,7 @@
         <v>CMY8GX3M2A1600C9A</v>
       </c>
       <c r="B844" t="str">
-        <v>Corsair Pro Series â 8GB</v>
+        <v>Corsair Pro Series — 8GB</v>
       </c>
       <c r="C844" t="str">
         <v>ram</v>
@@ -22349,7 +22349,7 @@
         <v>CMY8GX3M2A1600C9B</v>
       </c>
       <c r="B845" t="str">
-        <v>Corsair Pro Series â 8GB</v>
+        <v>Corsair Pro Series — 8GB</v>
       </c>
       <c r="C845" t="str">
         <v>ram</v>
@@ -22375,7 +22375,7 @@
         <v>CMY8GX3M2A1600C9R</v>
       </c>
       <c r="B846" t="str">
-        <v>Corsair Pro Series â 8GB</v>
+        <v>Corsair Pro Series — 8GB</v>
       </c>
       <c r="C846" t="str">
         <v>ram</v>
@@ -27289,7 +27289,7 @@
         <v>CMH32GX4M2Z3600C18</v>
       </c>
       <c r="B1035" t="str">
-        <v>Corsair Vengeance RGB Pro SL fÃ¼r AMD Ryzen</v>
+        <v>Corsair Vengeance RGB Pro SL für AMD Ryzen</v>
       </c>
       <c r="C1035" t="str">
         <v>ram</v>
@@ -27315,7 +27315,7 @@
         <v>CMH32GX4M2Z3200C16</v>
       </c>
       <c r="B1036" t="str">
-        <v>Corsair Vengeance RGB Pro SL fÃ¼r AMD Ryzen</v>
+        <v>Corsair Vengeance RGB Pro SL für AMD Ryzen</v>
       </c>
       <c r="C1036" t="str">
         <v>ram</v>
@@ -28199,7 +28199,7 @@
         <v>CMX4GX3M2A1600C9</v>
       </c>
       <c r="B1070" t="str">
-        <v>Corsair XMS DDR3-1600 CL9 fÃ¼r Core i5/i7</v>
+        <v>Corsair XMS DDR3-1600 CL9 für Core i5/i7</v>
       </c>
       <c r="C1070" t="str">
         <v>ram</v>
@@ -28303,7 +28303,7 @@
         <v>CMX4GX3M1A1333C9</v>
       </c>
       <c r="B1074" t="str">
-        <v>Corsair XMS3 DDR3-1333 CL9 fÃ¼r AMD/Core i3/i5/i7</v>
+        <v>Corsair XMS3 DDR3-1333 CL9 für AMD/Core i3/i5/i7</v>
       </c>
       <c r="C1074" t="str">
         <v>ram</v>
@@ -28355,7 +28355,7 @@
         <v>CMZ12GX3M3A2000C10</v>
       </c>
       <c r="B1076" t="str">
-        <v>Corsair â 12GB Triple Channel DDR3 Memory Kit</v>
+        <v>Corsair — 12GB Triple Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1076" t="str">
         <v>ram</v>
@@ -28381,7 +28381,7 @@
         <v>CMZ16GX3M2A1600C10B</v>
       </c>
       <c r="B1077" t="str">
-        <v>Corsair â 16GB Dual Channel DDR3 Memory Kit</v>
+        <v>Corsair — 16GB Dual Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1077" t="str">
         <v>ram</v>
@@ -28407,7 +28407,7 @@
         <v>CMZ24GX3M6A1600C9</v>
       </c>
       <c r="B1078" t="str">
-        <v>Corsair â 24GB Triple Channel DDR3 Memory Kit</v>
+        <v>Corsair — 24GB Triple Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1078" t="str">
         <v>ram</v>
@@ -28433,7 +28433,7 @@
         <v>CMZ32GX3M4X1600C10</v>
       </c>
       <c r="B1079" t="str">
-        <v>Corsair â 32GB Dual/Quad Channel DDR3 Memory Kit</v>
+        <v>Corsair — 32GB Dual/Quad Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1079" t="str">
         <v>ram</v>
@@ -28459,7 +28459,7 @@
         <v>CMZ4GX3M2A1600C9</v>
       </c>
       <c r="B1080" t="str">
-        <v>Corsair â 4GB Dual Channel DDR3 Memory Kit</v>
+        <v>Corsair — 4GB Dual Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1080" t="str">
         <v>ram</v>
@@ -28485,7 +28485,7 @@
         <v>CMZ4GX3M1A1600C9</v>
       </c>
       <c r="B1081" t="str">
-        <v>Corsair â 4GB Single Module DDR3 Memory Kit</v>
+        <v>Corsair — 4GB Single Module DDR3 Memory Kit</v>
       </c>
       <c r="C1081" t="str">
         <v>ram</v>
@@ -28511,7 +28511,7 @@
         <v>CMZ4GX3M1A1600C9B</v>
       </c>
       <c r="B1082" t="str">
-        <v>Corsair â 4GB Single Module DDR3 Memory Kit</v>
+        <v>Corsair — 4GB Single Module DDR3 Memory Kit</v>
       </c>
       <c r="C1082" t="str">
         <v>ram</v>
@@ -28537,7 +28537,7 @@
         <v>CMZ64GX3M8A1600C9</v>
       </c>
       <c r="B1083" t="str">
-        <v>Corsair â 64GB Quad Channel DDR3 Memory Kit</v>
+        <v>Corsair — 64GB Quad Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1083" t="str">
         <v>ram</v>
@@ -28563,7 +28563,7 @@
         <v>CMZ8GX3M1A1600C10B</v>
       </c>
       <c r="B1084" t="str">
-        <v>Corsair â 8GB DDR3 Memory Kit</v>
+        <v>Corsair — 8GB DDR3 Memory Kit</v>
       </c>
       <c r="C1084" t="str">
         <v>ram</v>
@@ -28589,7 +28589,7 @@
         <v>CMZ8GX3M2A1600C9B</v>
       </c>
       <c r="B1085" t="str">
-        <v>Corsair â 8GB Dual Channel DDR3 Memory Kit</v>
+        <v>Corsair — 8GB Dual Channel DDR3 Memory Kit</v>
       </c>
       <c r="C1085" t="str">
         <v>ram</v>
@@ -59035,7 +59035,7 @@
         <v>CC-9011095-WW</v>
       </c>
       <c r="B2256" t="str">
-        <v>Carbide Series Clear 400C Compact Mid-Tower â White</v>
+        <v>Carbide Series Clear 400C Compact Mid-Tower — White</v>
       </c>
       <c r="C2256" t="str">
         <v>case</v>
@@ -59165,7 +59165,7 @@
         <v>CC-9011085-WW</v>
       </c>
       <c r="B2261" t="str">
-        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming â Black/Red</v>
+        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming — Black/Red</v>
       </c>
       <c r="C2261" t="str">
         <v>case</v>
@@ -59191,7 +59191,7 @@
         <v>CC-9011084-WW</v>
       </c>
       <c r="B2262" t="str">
-        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming â Black/Silver</v>
+        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming — Black/Silver</v>
       </c>
       <c r="C2262" t="str">
         <v>case</v>
@@ -59217,7 +59217,7 @@
         <v>CC-9011094-WW</v>
       </c>
       <c r="B2263" t="str">
-        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming â Black/Yellow</v>
+        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming — Black/Yellow</v>
       </c>
       <c r="C2263" t="str">
         <v>case</v>
@@ -59243,7 +59243,7 @@
         <v>CC-9011083-WW</v>
       </c>
       <c r="B2264" t="str">
-        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming â White/Red</v>
+        <v>Carbide Series SPEC-ALPHA Mid-Tower Gaming — White/Red</v>
       </c>
       <c r="C2264" t="str">
         <v>case</v>
@@ -60985,7 +60985,7 @@
         <v>CC-9011129-WW</v>
       </c>
       <c r="B2331" t="str">
-        <v>Crystal Series 460X RGB Compact ATX Mid-Tower â White</v>
+        <v>Crystal Series 460X RGB Compact ATX Mid-Tower — White</v>
       </c>
       <c r="C2331" t="str">
         <v>case</v>
@@ -61037,7 +61037,7 @@
         <v>CC-9011111-WW</v>
       </c>
       <c r="B2333" t="str">
-        <v>Crystal Series 570X RGB ATX Mid-Tower â Red</v>
+        <v>Crystal Series 570X RGB ATX Mid-Tower — Red</v>
       </c>
       <c r="C2333" t="str">
         <v>case</v>
@@ -61063,7 +61063,7 @@
         <v>CC-9011110-WW</v>
       </c>
       <c r="B2334" t="str">
-        <v>Crystal Series 570X RGB ATX Mid-Tower â White</v>
+        <v>Crystal Series 570X RGB ATX Mid-Tower — White</v>
       </c>
       <c r="C2334" t="str">
         <v>case</v>
@@ -61193,7 +61193,7 @@
         <v>FD-C-DEF7A-03</v>
       </c>
       <c r="B2339" t="str">
-        <v>Fractal Design Define 7 Black Dark TG Midi-Tower - getÃ¶ntes Tempered Glass, isolated, black</v>
+        <v>Fractal Design Define 7 Black Dark TG Midi-Tower - getöntes Tempered Glass, isolated, black</v>
       </c>
       <c r="C2339" t="str">
         <v>case</v>
@@ -66107,7 +66107,7 @@
         <v>PH-ES813P_SGR</v>
       </c>
       <c r="B2528" t="str">
-        <v>PHANTEKS Enthoo Primo SE Big-Tower, grÃ¼ne LED - black/grÃ¼n</v>
+        <v>PHANTEKS Enthoo Primo SE Big-Tower, grüne LED - black/grün</v>
       </c>
       <c r="C2528" t="str">
         <v>case</v>
@@ -68603,7 +68603,7 @@
         <v>0-761345-10921-5</v>
       </c>
       <c r="B2624" t="str">
-        <v>Antec A400 RGB Processor KÃ¼hler</v>
+        <v>Antec A400 RGB Processor Kühler</v>
       </c>
       <c r="C2624" t="str">
         <v>cpu-cooler</v>
@@ -75170,7 +75170,7 @@
         <v/>
       </c>
       <c r="G2876" t="str">
-        <v>AOC. 28", 3840 Ã 2160, 60 Hz, TN, 1 ms, FreeSync</v>
+        <v>AOC. 28", 3840 × 2160, 60 Hz, TN, 1 ms, FreeSync</v>
       </c>
       <c r="H2876" t="str">
         <v>monitor,aoc</v>
@@ -75248,7 +75248,7 @@
         <v/>
       </c>
       <c r="G2879" t="str">
-        <v>ASUS. 28", 3840 Ã 2160, 60 Hz, TN, 1 ms</v>
+        <v>ASUS. 28", 3840 × 2160, 60 Hz, TN, 1 ms</v>
       </c>
       <c r="H2879" t="str">
         <v>monitor,asus</v>
@@ -75274,7 +75274,7 @@
         <v/>
       </c>
       <c r="G2880" t="str">
-        <v>ASUS. 27", 3840 Ã 2160, 144 Hz, IPS, 4 ms</v>
+        <v>ASUS. 27", 3840 × 2160, 144 Hz, IPS, 4 ms</v>
       </c>
       <c r="H2880" t="str">
         <v>monitor,asus,gaming</v>
@@ -75508,7 +75508,7 @@
         <v/>
       </c>
       <c r="G2889" t="str">
-        <v>ASUS. 28", 3840 Ã 2160, 60 Hz, IPS, 5 ms</v>
+        <v>ASUS. 28", 3840 × 2160, 60 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2889" t="str">
         <v>monitor,asus</v>
@@ -75820,7 +75820,7 @@
         <v/>
       </c>
       <c r="G2901" t="str">
-        <v>LG. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
+        <v>LG. 27", 3840 × 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
       </c>
       <c r="H2901" t="str">
         <v>monitor,lg</v>
@@ -75846,7 +75846,7 @@
         <v/>
       </c>
       <c r="G2902" t="str">
-        <v>LG. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
+        <v>LG. 27", 3840 × 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
       </c>
       <c r="H2902" t="str">
         <v>monitor,lg</v>
@@ -75872,7 +75872,7 @@
         <v/>
       </c>
       <c r="G2903" t="str">
-        <v>LG. 27", 3840 Ã 2160, 60 Hz, IPS, 4 ms, FreeSync</v>
+        <v>LG. 27", 3840 × 2160, 60 Hz, IPS, 4 ms, FreeSync</v>
       </c>
       <c r="H2903" t="str">
         <v>monitor,lg</v>
@@ -75924,7 +75924,7 @@
         <v/>
       </c>
       <c r="G2905" t="str">
-        <v>LG. 31.5", 3840 Ã 2160, 60 Hz, VA, 4 ms, FreeSync</v>
+        <v>LG. 31.5", 3840 × 2160, 60 Hz, VA, 4 ms, FreeSync</v>
       </c>
       <c r="H2905" t="str">
         <v>monitor,lg</v>
@@ -76054,7 +76054,7 @@
         <v/>
       </c>
       <c r="G2910" t="str">
-        <v>LG. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms</v>
+        <v>LG. 27", 3840 × 2160, 60 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2910" t="str">
         <v>monitor,lg</v>
@@ -76418,7 +76418,7 @@
         <v/>
       </c>
       <c r="G2924" t="str">
-        <v>ViewSonic. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms</v>
+        <v>ViewSonic. 27", 3840 × 2160, 60 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2924" t="str">
         <v>monitor,viewsonic</v>
@@ -76496,7 +76496,7 @@
         <v/>
       </c>
       <c r="G2927" t="str">
-        <v>ViewSonic. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms</v>
+        <v>ViewSonic. 27", 3840 × 2160, 60 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2927" t="str">
         <v>monitor,viewsonic</v>
@@ -76522,7 +76522,7 @@
         <v/>
       </c>
       <c r="G2928" t="str">
-        <v>ViewSonic. 32", 3840 Ã 2160, 122 Hz, IPS, 5 ms</v>
+        <v>ViewSonic. 32", 3840 × 2160, 122 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2928" t="str">
         <v>monitor,viewsonic</v>
@@ -76834,7 +76834,7 @@
         <v/>
       </c>
       <c r="G2940" t="str">
-        <v>ViewSonic. 27", 3840 Ã 2160, 60 Hz, IPS, 4 ms</v>
+        <v>ViewSonic. 27", 3840 × 2160, 60 Hz, IPS, 4 ms</v>
       </c>
       <c r="H2940" t="str">
         <v>monitor,viewsonic</v>
@@ -76938,7 +76938,7 @@
         <v/>
       </c>
       <c r="G2944" t="str">
-        <v>ViewSonic. 32", 3840 Ã 2160, 60 Hz, VA, 3 ms, FreeSync</v>
+        <v>ViewSonic. 32", 3840 × 2160, 60 Hz, VA, 3 ms, FreeSync</v>
       </c>
       <c r="H2944" t="str">
         <v>monitor,viewsonic</v>
@@ -77068,7 +77068,7 @@
         <v/>
       </c>
       <c r="G2949" t="str">
-        <v>ViewSonic. 31.5", 3840 Ã 2160, 60 Hz, VA, 4 ms</v>
+        <v>ViewSonic. 31.5", 3840 × 2160, 60 Hz, VA, 4 ms</v>
       </c>
       <c r="H2949" t="str">
         <v>monitor,viewsonic</v>
@@ -77120,7 +77120,7 @@
         <v/>
       </c>
       <c r="G2951" t="str">
-        <v>ViewSonic. 43", 3840 Ã 2160, 60 Hz, IPS, 5 ms</v>
+        <v>ViewSonic. 43", 3840 × 2160, 60 Hz, IPS, 5 ms</v>
       </c>
       <c r="H2951" t="str">
         <v>monitor,viewsonic</v>
@@ -77224,7 +77224,7 @@
         <v/>
       </c>
       <c r="G2955" t="str">
-        <v>ViewSonic. 27", 3840 Ã 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
+        <v>ViewSonic. 27", 3840 × 2160, 60 Hz, IPS, 5 ms, FreeSync</v>
       </c>
       <c r="H2955" t="str">
         <v>monitor,viewsonic</v>
@@ -77354,7 +77354,7 @@
         <v/>
       </c>
       <c r="G2960" t="str">
-        <v>ViewSonic. 32", 3840 Ã 2160, 144 Hz, IPS, Quantum Dot, 1 ms</v>
+        <v>ViewSonic. 32", 3840 × 2160, 144 Hz, IPS, Quantum Dot, 1 ms</v>
       </c>
       <c r="H2960" t="str">
         <v>monitor,viewsonic,gaming</v>
@@ -77380,7 +77380,7 @@
         <v/>
       </c>
       <c r="G2961" t="str">
-        <v>ViewSonic. 32", 3840 Ã 2160, 60 Hz, VA, 5 ms</v>
+        <v>ViewSonic. 32", 3840 × 2160, 60 Hz, VA, 5 ms</v>
       </c>
       <c r="H2961" t="str">
         <v>monitor,viewsonic</v>

</xml_diff>